<commit_message>
feat: update bulk templates and remove DisplayOrderDrawer component; enhance admin API for reviews
</commit_message>
<xml_diff>
--- a/public/templates/2_Litmus_Tests_Bulk_Template.xlsx
+++ b/public/templates/2_Litmus_Tests_Bulk_Template.xlsx
@@ -488,10 +488,10 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:Q7"/>
+  <dimension ref="A1:R7"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15" outlineLevelCol="0"/>
   <cols>
-    <col width="148" customWidth="1" min="1" max="1"/>
+    <col width="231" customWidth="1" min="1" max="1"/>
     <col width="14" customWidth="1" min="2" max="2"/>
     <col width="16" customWidth="1" min="3" max="3"/>
     <col width="17" customWidth="1" min="4" max="4"/>
@@ -508,12 +508,13 @@
     <col width="30" customWidth="1" min="15" max="15"/>
     <col width="14" customWidth="1" min="16" max="16"/>
     <col width="121" customWidth="1" min="17" max="17"/>
+    <col width="16" customWidth="1" min="18" max="18"/>
   </cols>
   <sheetData>
     <row r="1" ht="28" customHeight="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>INSTRUCTIONS: Define test details, optional subcategories, and parameters. Use 'Name:Unit:Min:Max:Price' format for parameters separated by ';'.</t>
+          <t>INSTRUCTIONS: Define test details, optional subcategories, and parameters. Use 'Name:Unit:Min:Max:Price' format for parameters separated by ';'. Optional 'displayOrder' sets the website priority (1 = shown first; 0 removes it).</t>
         </is>
       </c>
     </row>
@@ -603,6 +604,11 @@
           <t>parameters</t>
         </is>
       </c>
+      <c r="R2" s="2" t="inlineStr">
+        <is>
+          <t>displayOrder</t>
+        </is>
+      </c>
     </row>
     <row r="3" ht="18" customHeight="1">
       <c r="A3" s="3" t="inlineStr">
@@ -690,6 +696,11 @@
           <t>OPTIONAL</t>
         </is>
       </c>
+      <c r="R3" s="4" t="inlineStr">
+        <is>
+          <t>OPTIONAL</t>
+        </is>
+      </c>
     </row>
     <row r="4" ht="22" customHeight="1">
       <c r="A4" s="5" t="inlineStr">
@@ -767,6 +778,9 @@
           <t>Total Fat:%:3.0:8.0:180; Solids Not Fat (SNF):%:8.0:10.5:120; Density:g/ml:1.026:1.032:100</t>
         </is>
       </c>
+      <c r="R4" s="5" t="n">
+        <v>1</v>
+      </c>
     </row>
     <row r="5" ht="22" customHeight="1">
       <c r="A5" s="5" t="inlineStr">
@@ -840,6 +854,9 @@
           <t>Moisture Content:%:0:60.0:250; Fat on Dry Basis:%:45.0:70.0:300</t>
         </is>
       </c>
+      <c r="R5" s="5" t="n">
+        <v>2</v>
+      </c>
     </row>
     <row r="6" ht="22" customHeight="1">
       <c r="A6" s="5" t="inlineStr">
@@ -905,6 +922,7 @@
           <t>Total Coliform Count:cfu/g:0:10:350; E. Coli Count:cfu/g:0:0:450</t>
         </is>
       </c>
+      <c r="R6" s="5" t="inlineStr"/>
     </row>
     <row r="7" ht="22" customHeight="1">
       <c r="A7" s="5" t="inlineStr">
@@ -970,10 +988,11 @@
           <t>Lead (Pb):ppm:0.0:0.1:400; Cadmium (Cd):ppm:0.0:0.05:400; Arsenic (As):ppm:0.0:0.1:450; Mercury (Hg):ppm:0.0:0.01:450</t>
         </is>
       </c>
+      <c r="R7" s="5" t="inlineStr"/>
     </row>
   </sheetData>
   <mergeCells count="1">
-    <mergeCell ref="A1:Q1"/>
+    <mergeCell ref="A1:R1"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>